<commit_message>
Name the Race #09 ninth-place rider and keep teams per race
The updated results sheet fills in bib 247, who finished ninth in Elite
in 1:33:57.42 and was previously listed only as a placeholder. They are
Aira Saran of HAMMERDOWN COACHING, already a known rider, so the result
attaches to their existing profile and counts towards their record.
Nothing else in the sheet changed.

Results also keep the team the rider actually rode for. The team was read
from each race sheet and then thrown away, so results borrowed whatever
team the rider is currently listed under — four of the nine Elite
finishers here showed as DELTA Team when the sheet says HAMMERDOWN
COACHING. Results now carry their own team and fall back to the rider's
current one only when the sheet recorded none. This corrects 646 rows
across the archive.
</commit_message>
<xml_diff>
--- a/public/2026 results/BBCh26Race09Results.xlsx
+++ b/public/2026 results/BBCh26Race09Results.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\124329\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Promise\My Data\#Events\BBCh\2026\Race #09 - XC &amp; Trail Run\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C39AE046-976B-DB47-B0E0-19EC9156C2CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CBB19C9-4CD8-44A4-AE68-7208D795A04B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{0FA67269-9C1A-416D-BF45-AC14718C6D2A}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{0FA67269-9C1A-416D-BF45-AC14718C6D2A}"/>
   </bookViews>
   <sheets>
     <sheet name="Results" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="335" uniqueCount="270">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="335" uniqueCount="269">
   <si>
     <t>Elite</t>
   </si>
@@ -302,9 +302,6 @@
     <t>1:32:16.77</t>
   </si>
   <si>
-    <t>ZE Dummy 01</t>
-  </si>
-  <si>
     <t>0:12:11.54</t>
   </si>
   <si>
@@ -846,6 +843,9 @@
   </si>
   <si>
     <t>Yohaan Sarda</t>
+  </si>
+  <si>
+    <t>Aira Saran</t>
   </si>
 </sst>
 </file>
@@ -1451,18 +1451,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9120722D-0728-4F6A-BA31-4B000BFC76BB}">
   <dimension ref="C3:M52"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="3" width="6.05078125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="23.5390625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="23.9453125" bestFit="1" customWidth="1"/>
-    <col min="6" max="8" width="9.68359375" bestFit="1" customWidth="1"/>
-    <col min="9" max="11" width="11.56640625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="9.68359375" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="11.56640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="6" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="23.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="24" bestFit="1" customWidth="1"/>
+    <col min="6" max="8" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="11" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="3:13" x14ac:dyDescent="0.2">
+    <row r="3" spans="3:13" x14ac:dyDescent="0.25">
       <c r="C3" s="2" t="s">
         <v>0</v>
       </c>
@@ -1477,7 +1477,7 @@
       <c r="L3" s="3"/>
       <c r="M3" s="3"/>
     </row>
-    <row r="4" spans="3:13" x14ac:dyDescent="0.2">
+    <row r="4" spans="3:13" x14ac:dyDescent="0.25">
       <c r="C4" t="s">
         <v>1</v>
       </c>
@@ -1512,7 +1512,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="3:13" x14ac:dyDescent="0.2">
+    <row r="5" spans="3:13" x14ac:dyDescent="0.25">
       <c r="C5">
         <v>215</v>
       </c>
@@ -1547,7 +1547,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="3:13" x14ac:dyDescent="0.2">
+    <row r="6" spans="3:13" x14ac:dyDescent="0.25">
       <c r="C6">
         <v>235</v>
       </c>
@@ -1582,7 +1582,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="7" spans="3:13" x14ac:dyDescent="0.2">
+    <row r="7" spans="3:13" x14ac:dyDescent="0.25">
       <c r="C7">
         <v>237</v>
       </c>
@@ -1617,7 +1617,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="8" spans="3:13" x14ac:dyDescent="0.2">
+    <row r="8" spans="3:13" x14ac:dyDescent="0.25">
       <c r="C8">
         <v>246</v>
       </c>
@@ -1652,7 +1652,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="9" spans="3:13" x14ac:dyDescent="0.2">
+    <row r="9" spans="3:13" x14ac:dyDescent="0.25">
       <c r="C9">
         <v>221</v>
       </c>
@@ -1687,7 +1687,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="10" spans="3:13" x14ac:dyDescent="0.2">
+    <row r="10" spans="3:13" x14ac:dyDescent="0.25">
       <c r="C10">
         <v>222</v>
       </c>
@@ -1722,7 +1722,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="11" spans="3:13" x14ac:dyDescent="0.2">
+    <row r="11" spans="3:13" x14ac:dyDescent="0.25">
       <c r="C11">
         <v>245</v>
       </c>
@@ -1757,7 +1757,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="12" spans="3:13" x14ac:dyDescent="0.2">
+    <row r="12" spans="3:13" x14ac:dyDescent="0.25">
       <c r="C12">
         <v>233</v>
       </c>
@@ -1792,44 +1792,44 @@
         <v>86</v>
       </c>
     </row>
-    <row r="13" spans="3:13" x14ac:dyDescent="0.2">
+    <row r="13" spans="3:13" x14ac:dyDescent="0.25">
       <c r="C13">
         <v>247</v>
       </c>
       <c r="D13" t="s">
+        <v>268</v>
+      </c>
+      <c r="E13" t="s">
+        <v>23</v>
+      </c>
+      <c r="F13" t="s">
         <v>87</v>
       </c>
-      <c r="E13" t="s">
-        <v>60</v>
-      </c>
-      <c r="F13" t="s">
+      <c r="G13" t="s">
         <v>88</v>
       </c>
-      <c r="G13" t="s">
+      <c r="H13" t="s">
         <v>89</v>
       </c>
-      <c r="H13" t="s">
+      <c r="I13" t="s">
         <v>90</v>
       </c>
-      <c r="I13" t="s">
+      <c r="J13" t="s">
         <v>91</v>
       </c>
-      <c r="J13" t="s">
+      <c r="K13" t="s">
         <v>92</v>
       </c>
-      <c r="K13" t="s">
+      <c r="L13" t="s">
         <v>93</v>
       </c>
-      <c r="L13" t="s">
+      <c r="M13" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="M13" s="1" t="s">
+    </row>
+    <row r="15" spans="3:13" x14ac:dyDescent="0.25">
+      <c r="C15" s="4" t="s">
         <v>95</v>
-      </c>
-    </row>
-    <row r="15" spans="3:13" x14ac:dyDescent="0.2">
-      <c r="C15" s="4" t="s">
-        <v>96</v>
       </c>
       <c r="D15" s="4"/>
       <c r="E15" s="4"/>
@@ -1839,7 +1839,7 @@
       <c r="I15" s="4"/>
       <c r="J15" s="4"/>
     </row>
-    <row r="16" spans="3:13" x14ac:dyDescent="0.2">
+    <row r="16" spans="3:13" x14ac:dyDescent="0.25">
       <c r="C16" t="s">
         <v>1</v>
       </c>
@@ -1865,419 +1865,419 @@
         <v>11</v>
       </c>
     </row>
-    <row r="17" spans="3:10" x14ac:dyDescent="0.2">
+    <row r="17" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C17">
         <v>323</v>
       </c>
       <c r="D17" t="s">
+        <v>96</v>
+      </c>
+      <c r="E17" t="s">
+        <v>60</v>
+      </c>
+      <c r="F17" t="s">
         <v>97</v>
       </c>
-      <c r="E17" t="s">
-        <v>60</v>
-      </c>
-      <c r="F17" t="s">
+      <c r="G17" t="s">
         <v>98</v>
       </c>
-      <c r="G17" t="s">
+      <c r="H17" t="s">
         <v>99</v>
       </c>
-      <c r="H17" t="s">
+      <c r="I17" t="s">
         <v>100</v>
       </c>
-      <c r="I17" t="s">
+      <c r="J17" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="J17" s="1" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="18" spans="3:10" x14ac:dyDescent="0.2">
+    </row>
+    <row r="18" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C18">
         <v>328</v>
       </c>
       <c r="D18" t="s">
+        <v>102</v>
+      </c>
+      <c r="E18" t="s">
+        <v>60</v>
+      </c>
+      <c r="F18" t="s">
         <v>103</v>
       </c>
-      <c r="E18" t="s">
-        <v>60</v>
-      </c>
-      <c r="F18" t="s">
+      <c r="G18" t="s">
         <v>104</v>
       </c>
-      <c r="G18" t="s">
+      <c r="H18" t="s">
         <v>105</v>
       </c>
-      <c r="H18" t="s">
+      <c r="I18" t="s">
         <v>106</v>
       </c>
-      <c r="I18" t="s">
+      <c r="J18" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="J18" s="1" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="19" spans="3:10" x14ac:dyDescent="0.2">
+    </row>
+    <row r="19" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C19">
         <v>339</v>
       </c>
       <c r="D19" t="s">
+        <v>108</v>
+      </c>
+      <c r="E19" t="s">
+        <v>60</v>
+      </c>
+      <c r="F19" t="s">
         <v>109</v>
       </c>
-      <c r="E19" t="s">
-        <v>60</v>
-      </c>
-      <c r="F19" t="s">
+      <c r="G19" t="s">
         <v>110</v>
       </c>
-      <c r="G19" t="s">
+      <c r="H19" t="s">
         <v>111</v>
       </c>
-      <c r="H19" t="s">
+      <c r="I19" t="s">
         <v>112</v>
       </c>
-      <c r="I19" t="s">
+      <c r="J19" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="J19" s="1" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="20" spans="3:10" x14ac:dyDescent="0.2">
+    </row>
+    <row r="20" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C20">
         <v>329</v>
       </c>
       <c r="D20" t="s">
+        <v>114</v>
+      </c>
+      <c r="E20" t="s">
+        <v>60</v>
+      </c>
+      <c r="F20" t="s">
         <v>115</v>
       </c>
-      <c r="E20" t="s">
-        <v>60</v>
-      </c>
-      <c r="F20" t="s">
+      <c r="G20" t="s">
         <v>116</v>
       </c>
-      <c r="G20" t="s">
+      <c r="H20" t="s">
         <v>117</v>
       </c>
-      <c r="H20" t="s">
+      <c r="I20" t="s">
         <v>118</v>
       </c>
-      <c r="I20" t="s">
+      <c r="J20" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="J20" s="1" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="21" spans="3:10" x14ac:dyDescent="0.2">
+    </row>
+    <row r="21" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C21">
         <v>340</v>
       </c>
       <c r="D21" t="s">
+        <v>120</v>
+      </c>
+      <c r="E21" t="s">
         <v>121</v>
       </c>
-      <c r="E21" t="s">
+      <c r="F21" t="s">
         <v>122</v>
       </c>
-      <c r="F21" t="s">
+      <c r="G21" t="s">
         <v>123</v>
       </c>
-      <c r="G21" t="s">
+      <c r="H21" t="s">
         <v>124</v>
       </c>
-      <c r="H21" t="s">
+      <c r="I21" t="s">
         <v>125</v>
       </c>
-      <c r="I21" t="s">
+      <c r="J21" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="J21" s="1" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="22" spans="3:10" x14ac:dyDescent="0.2">
+    </row>
+    <row r="22" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C22">
         <v>325</v>
       </c>
       <c r="D22" t="s">
+        <v>127</v>
+      </c>
+      <c r="E22" t="s">
+        <v>60</v>
+      </c>
+      <c r="F22" t="s">
         <v>128</v>
       </c>
-      <c r="E22" t="s">
-        <v>60</v>
-      </c>
-      <c r="F22" t="s">
+      <c r="G22" t="s">
         <v>129</v>
       </c>
-      <c r="G22" t="s">
+      <c r="H22" t="s">
         <v>130</v>
       </c>
-      <c r="H22" t="s">
+      <c r="I22" t="s">
         <v>131</v>
       </c>
-      <c r="I22" t="s">
+      <c r="J22" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="J22" s="1" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="23" spans="3:10" x14ac:dyDescent="0.2">
+    </row>
+    <row r="23" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C23">
         <v>324</v>
       </c>
       <c r="D23" t="s">
+        <v>133</v>
+      </c>
+      <c r="E23" t="s">
+        <v>60</v>
+      </c>
+      <c r="F23" t="s">
         <v>134</v>
       </c>
-      <c r="E23" t="s">
-        <v>60</v>
-      </c>
-      <c r="F23" t="s">
+      <c r="G23" t="s">
         <v>135</v>
       </c>
-      <c r="G23" t="s">
+      <c r="H23" t="s">
         <v>136</v>
       </c>
-      <c r="H23" t="s">
+      <c r="I23" t="s">
         <v>137</v>
       </c>
-      <c r="I23" t="s">
+      <c r="J23" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="J23" s="1" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="24" spans="3:10" x14ac:dyDescent="0.2">
+    </row>
+    <row r="24" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C24">
         <v>330</v>
       </c>
       <c r="D24" t="s">
+        <v>139</v>
+      </c>
+      <c r="E24" t="s">
+        <v>60</v>
+      </c>
+      <c r="F24" t="s">
         <v>140</v>
       </c>
-      <c r="E24" t="s">
-        <v>60</v>
-      </c>
-      <c r="F24" t="s">
+      <c r="G24" t="s">
         <v>141</v>
       </c>
-      <c r="G24" t="s">
+      <c r="H24" t="s">
         <v>142</v>
       </c>
-      <c r="H24" t="s">
+      <c r="I24" t="s">
         <v>143</v>
       </c>
-      <c r="I24" t="s">
+      <c r="J24" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="J24" s="1" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="25" spans="3:10" x14ac:dyDescent="0.2">
+    </row>
+    <row r="25" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C25">
         <v>320</v>
       </c>
       <c r="D25" t="s">
+        <v>145</v>
+      </c>
+      <c r="E25" t="s">
+        <v>60</v>
+      </c>
+      <c r="F25" t="s">
         <v>146</v>
       </c>
-      <c r="E25" t="s">
-        <v>60</v>
-      </c>
-      <c r="F25" t="s">
+      <c r="G25" t="s">
         <v>147</v>
       </c>
-      <c r="G25" t="s">
+      <c r="H25" t="s">
         <v>148</v>
       </c>
-      <c r="H25" t="s">
+      <c r="I25" t="s">
         <v>149</v>
       </c>
-      <c r="I25" t="s">
+      <c r="J25" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="J25" s="1" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="26" spans="3:10" x14ac:dyDescent="0.2">
+    </row>
+    <row r="26" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C26">
         <v>335</v>
       </c>
       <c r="D26" t="s">
+        <v>151</v>
+      </c>
+      <c r="E26" t="s">
+        <v>60</v>
+      </c>
+      <c r="F26" t="s">
         <v>152</v>
       </c>
-      <c r="E26" t="s">
-        <v>60</v>
-      </c>
-      <c r="F26" t="s">
+      <c r="G26" t="s">
         <v>153</v>
       </c>
-      <c r="G26" t="s">
+      <c r="H26" t="s">
         <v>154</v>
       </c>
-      <c r="H26" t="s">
+      <c r="I26" t="s">
         <v>155</v>
       </c>
-      <c r="I26" t="s">
+      <c r="J26" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="J26" s="1" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="27" spans="3:10" x14ac:dyDescent="0.2">
+    </row>
+    <row r="27" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C27">
         <v>341</v>
       </c>
       <c r="D27" t="s">
+        <v>157</v>
+      </c>
+      <c r="E27" t="s">
+        <v>60</v>
+      </c>
+      <c r="F27" t="s">
         <v>158</v>
       </c>
-      <c r="E27" t="s">
-        <v>60</v>
-      </c>
-      <c r="F27" t="s">
+      <c r="G27" t="s">
         <v>159</v>
       </c>
-      <c r="G27" t="s">
+      <c r="H27" t="s">
         <v>160</v>
       </c>
-      <c r="H27" t="s">
+      <c r="I27" t="s">
         <v>161</v>
       </c>
-      <c r="I27" t="s">
+      <c r="J27" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="J27" s="1" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="28" spans="3:10" x14ac:dyDescent="0.2">
+    </row>
+    <row r="28" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C28">
         <v>336</v>
       </c>
       <c r="D28" t="s">
+        <v>163</v>
+      </c>
+      <c r="E28" t="s">
+        <v>60</v>
+      </c>
+      <c r="F28" t="s">
         <v>164</v>
       </c>
-      <c r="E28" t="s">
-        <v>60</v>
-      </c>
-      <c r="F28" t="s">
+      <c r="G28" t="s">
         <v>165</v>
       </c>
-      <c r="G28" t="s">
+      <c r="H28" t="s">
         <v>166</v>
       </c>
-      <c r="H28" t="s">
+      <c r="I28" t="s">
         <v>167</v>
       </c>
-      <c r="I28" t="s">
+      <c r="J28" s="1" t="s">
         <v>168</v>
       </c>
-      <c r="J28" s="1" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="29" spans="3:10" x14ac:dyDescent="0.2">
+    </row>
+    <row r="29" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C29">
         <v>319</v>
       </c>
       <c r="D29" t="s">
+        <v>169</v>
+      </c>
+      <c r="E29" t="s">
+        <v>60</v>
+      </c>
+      <c r="F29" t="s">
         <v>170</v>
       </c>
-      <c r="E29" t="s">
-        <v>60</v>
-      </c>
-      <c r="F29" t="s">
+      <c r="G29" t="s">
         <v>171</v>
       </c>
-      <c r="G29" t="s">
+      <c r="H29" t="s">
         <v>172</v>
       </c>
-      <c r="H29" t="s">
+      <c r="I29" t="s">
         <v>173</v>
       </c>
-      <c r="I29" t="s">
+      <c r="J29" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="J29" s="1" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="30" spans="3:10" x14ac:dyDescent="0.2">
+    </row>
+    <row r="30" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C30">
         <v>342</v>
       </c>
       <c r="D30" t="s">
+        <v>175</v>
+      </c>
+      <c r="E30" t="s">
+        <v>60</v>
+      </c>
+      <c r="F30" t="s">
         <v>176</v>
       </c>
-      <c r="E30" t="s">
-        <v>60</v>
-      </c>
-      <c r="F30" t="s">
+      <c r="G30" t="s">
         <v>177</v>
       </c>
-      <c r="G30" t="s">
+      <c r="H30" t="s">
         <v>178</v>
       </c>
-      <c r="H30" t="s">
+      <c r="I30" t="s">
         <v>179</v>
       </c>
-      <c r="I30" t="s">
+      <c r="J30" s="1" t="s">
         <v>180</v>
       </c>
-      <c r="J30" s="1" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="31" spans="3:10" x14ac:dyDescent="0.2">
+    </row>
+    <row r="31" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C31">
         <v>343</v>
       </c>
       <c r="D31" t="s">
+        <v>181</v>
+      </c>
+      <c r="E31" t="s">
+        <v>60</v>
+      </c>
+      <c r="F31" t="s">
         <v>182</v>
       </c>
-      <c r="E31" t="s">
-        <v>60</v>
-      </c>
-      <c r="F31" t="s">
+      <c r="G31" t="s">
         <v>183</v>
       </c>
-      <c r="G31" t="s">
+      <c r="H31" t="s">
         <v>184</v>
       </c>
-      <c r="H31" t="s">
+      <c r="I31" t="s">
         <v>185</v>
       </c>
-      <c r="I31" t="s">
+      <c r="J31" s="1" t="s">
         <v>186</v>
       </c>
-      <c r="J31" s="1" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="32" spans="3:10" x14ac:dyDescent="0.2">
+    </row>
+    <row r="32" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C32">
         <v>334</v>
       </c>
       <c r="D32" t="s">
+        <v>187</v>
+      </c>
+      <c r="E32" t="s">
+        <v>60</v>
+      </c>
+      <c r="F32" t="s">
         <v>188</v>
       </c>
-      <c r="E32" t="s">
-        <v>60</v>
-      </c>
-      <c r="F32" t="s">
+      <c r="G32" t="s">
         <v>189</v>
       </c>
-      <c r="G32" t="s">
+      <c r="J32" s="1" t="s">
         <v>190</v>
       </c>
-      <c r="J32" s="1" t="s">
+    </row>
+    <row r="34" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C34" s="5" t="s">
         <v>191</v>
-      </c>
-    </row>
-    <row r="34" spans="3:11" x14ac:dyDescent="0.2">
-      <c r="C34" s="5" t="s">
-        <v>192</v>
       </c>
       <c r="D34" s="6"/>
       <c r="E34" s="6"/>
@@ -2286,7 +2286,7 @@
       <c r="H34" s="6"/>
       <c r="I34" s="6"/>
     </row>
-    <row r="35" spans="3:11" x14ac:dyDescent="0.2">
+    <row r="35" spans="3:11" x14ac:dyDescent="0.25">
       <c r="C35" t="s">
         <v>1</v>
       </c>
@@ -2309,193 +2309,193 @@
         <v>11</v>
       </c>
     </row>
-    <row r="36" spans="3:11" x14ac:dyDescent="0.2">
+    <row r="36" spans="3:11" x14ac:dyDescent="0.25">
       <c r="C36">
         <v>605</v>
       </c>
       <c r="D36" t="s">
+        <v>192</v>
+      </c>
+      <c r="E36" t="s">
         <v>193</v>
       </c>
-      <c r="E36" t="s">
+      <c r="F36" t="s">
         <v>194</v>
       </c>
-      <c r="F36" t="s">
+      <c r="G36" t="s">
         <v>195</v>
       </c>
-      <c r="G36" t="s">
+      <c r="H36" t="s">
         <v>196</v>
       </c>
-      <c r="H36" t="s">
+      <c r="I36" s="1" t="s">
         <v>197</v>
       </c>
-      <c r="I36" s="1" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="37" spans="3:11" x14ac:dyDescent="0.2">
+    </row>
+    <row r="37" spans="3:11" x14ac:dyDescent="0.25">
       <c r="C37">
         <v>612</v>
       </c>
       <c r="D37" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="E37" t="s">
         <v>60</v>
       </c>
       <c r="F37" t="s">
+        <v>198</v>
+      </c>
+      <c r="G37" t="s">
         <v>199</v>
       </c>
-      <c r="G37" t="s">
+      <c r="H37" t="s">
         <v>200</v>
       </c>
-      <c r="H37" t="s">
+      <c r="I37" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="I37" s="1" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="38" spans="3:11" x14ac:dyDescent="0.2">
+    </row>
+    <row r="38" spans="3:11" x14ac:dyDescent="0.25">
       <c r="C38">
         <v>607</v>
       </c>
       <c r="D38" t="s">
+        <v>202</v>
+      </c>
+      <c r="E38" t="s">
+        <v>60</v>
+      </c>
+      <c r="F38" t="s">
         <v>203</v>
       </c>
-      <c r="E38" t="s">
-        <v>60</v>
-      </c>
-      <c r="F38" t="s">
+      <c r="G38" t="s">
         <v>204</v>
       </c>
-      <c r="G38" t="s">
+      <c r="H38" t="s">
         <v>205</v>
       </c>
-      <c r="H38" t="s">
+      <c r="I38" s="1" t="s">
         <v>206</v>
       </c>
-      <c r="I38" s="1" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="39" spans="3:11" x14ac:dyDescent="0.2">
+    </row>
+    <row r="39" spans="3:11" x14ac:dyDescent="0.25">
       <c r="C39">
         <v>611</v>
       </c>
       <c r="D39" t="s">
+        <v>207</v>
+      </c>
+      <c r="E39" t="s">
+        <v>60</v>
+      </c>
+      <c r="F39" t="s">
         <v>208</v>
       </c>
-      <c r="E39" t="s">
-        <v>60</v>
-      </c>
-      <c r="F39" t="s">
+      <c r="G39" t="s">
         <v>209</v>
       </c>
-      <c r="G39" t="s">
+      <c r="H39" t="s">
         <v>210</v>
       </c>
-      <c r="H39" t="s">
+      <c r="I39" s="1" t="s">
         <v>211</v>
       </c>
-      <c r="I39" s="1" t="s">
-        <v>212</v>
-      </c>
-    </row>
-    <row r="40" spans="3:11" x14ac:dyDescent="0.2">
+    </row>
+    <row r="40" spans="3:11" x14ac:dyDescent="0.25">
       <c r="C40">
         <v>603</v>
       </c>
       <c r="D40" t="s">
+        <v>212</v>
+      </c>
+      <c r="E40" t="s">
+        <v>60</v>
+      </c>
+      <c r="F40" t="s">
         <v>213</v>
       </c>
-      <c r="E40" t="s">
-        <v>60</v>
-      </c>
-      <c r="F40" t="s">
+      <c r="G40" t="s">
         <v>214</v>
       </c>
-      <c r="G40" t="s">
+      <c r="H40" t="s">
         <v>215</v>
       </c>
-      <c r="H40" t="s">
+      <c r="I40" s="1" t="s">
         <v>216</v>
       </c>
-      <c r="I40" s="1" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="41" spans="3:11" x14ac:dyDescent="0.2">
+    </row>
+    <row r="41" spans="3:11" x14ac:dyDescent="0.25">
       <c r="C41">
         <v>601</v>
       </c>
       <c r="D41" t="s">
+        <v>217</v>
+      </c>
+      <c r="E41" t="s">
+        <v>60</v>
+      </c>
+      <c r="F41" t="s">
         <v>218</v>
       </c>
-      <c r="E41" t="s">
-        <v>60</v>
-      </c>
-      <c r="F41" t="s">
+      <c r="G41" t="s">
         <v>219</v>
       </c>
-      <c r="G41" t="s">
+      <c r="H41" t="s">
         <v>220</v>
       </c>
-      <c r="H41" t="s">
+      <c r="I41" s="1" t="s">
         <v>221</v>
       </c>
-      <c r="I41" s="1" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="42" spans="3:11" x14ac:dyDescent="0.2">
+    </row>
+    <row r="42" spans="3:11" x14ac:dyDescent="0.25">
       <c r="C42">
         <v>602</v>
       </c>
       <c r="D42" t="s">
+        <v>222</v>
+      </c>
+      <c r="E42" t="s">
+        <v>60</v>
+      </c>
+      <c r="F42" t="s">
         <v>223</v>
       </c>
-      <c r="E42" t="s">
-        <v>60</v>
-      </c>
-      <c r="F42" t="s">
+      <c r="G42" t="s">
         <v>224</v>
       </c>
-      <c r="G42" t="s">
+      <c r="H42" t="s">
         <v>225</v>
       </c>
-      <c r="H42" t="s">
+      <c r="I42" s="1" t="s">
         <v>226</v>
       </c>
-      <c r="I42" s="1" t="s">
-        <v>227</v>
-      </c>
-    </row>
-    <row r="43" spans="3:11" x14ac:dyDescent="0.2">
+    </row>
+    <row r="43" spans="3:11" x14ac:dyDescent="0.25">
       <c r="C43">
         <v>606</v>
       </c>
       <c r="D43" t="s">
+        <v>227</v>
+      </c>
+      <c r="E43" t="s">
+        <v>60</v>
+      </c>
+      <c r="F43" t="s">
         <v>228</v>
       </c>
-      <c r="E43" t="s">
-        <v>60</v>
-      </c>
-      <c r="F43" t="s">
+      <c r="G43" t="s">
         <v>229</v>
       </c>
-      <c r="G43" t="s">
+      <c r="H43" t="s">
         <v>230</v>
       </c>
-      <c r="H43" t="s">
+      <c r="I43" s="1" t="s">
         <v>231</v>
       </c>
-      <c r="I43" s="1" t="s">
+    </row>
+    <row r="45" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C45" s="7" t="s">
         <v>232</v>
-      </c>
-    </row>
-    <row r="45" spans="3:11" x14ac:dyDescent="0.2">
-      <c r="C45" s="7" t="s">
-        <v>233</v>
       </c>
       <c r="D45" s="8"/>
       <c r="E45" s="8"/>
@@ -2506,7 +2506,7 @@
       <c r="J45" s="8"/>
       <c r="K45" s="8"/>
     </row>
-    <row r="46" spans="3:11" x14ac:dyDescent="0.2">
+    <row r="46" spans="3:11" x14ac:dyDescent="0.25">
       <c r="C46" t="s">
         <v>1</v>
       </c>
@@ -2535,178 +2535,178 @@
         <v>11</v>
       </c>
     </row>
-    <row r="47" spans="3:11" x14ac:dyDescent="0.2">
+    <row r="47" spans="3:11" x14ac:dyDescent="0.25">
       <c r="C47">
         <v>28</v>
       </c>
       <c r="D47" t="s">
+        <v>233</v>
+      </c>
+      <c r="E47" t="s">
+        <v>60</v>
+      </c>
+      <c r="F47" t="s">
         <v>234</v>
       </c>
-      <c r="E47" t="s">
-        <v>60</v>
-      </c>
-      <c r="F47" t="s">
+      <c r="G47" t="s">
         <v>235</v>
       </c>
-      <c r="G47" t="s">
+      <c r="H47" t="s">
         <v>236</v>
       </c>
-      <c r="H47" t="s">
+      <c r="I47" t="s">
         <v>237</v>
       </c>
-      <c r="I47" t="s">
+      <c r="J47" t="s">
         <v>238</v>
       </c>
-      <c r="J47" t="s">
+      <c r="K47" s="1" t="s">
         <v>239</v>
       </c>
-      <c r="K47" s="1" t="s">
-        <v>240</v>
-      </c>
-    </row>
-    <row r="48" spans="3:11" x14ac:dyDescent="0.2">
+    </row>
+    <row r="48" spans="3:11" x14ac:dyDescent="0.25">
       <c r="C48">
         <v>10</v>
       </c>
       <c r="D48" t="s">
+        <v>240</v>
+      </c>
+      <c r="E48" t="s">
+        <v>60</v>
+      </c>
+      <c r="F48" t="s">
         <v>241</v>
       </c>
-      <c r="E48" t="s">
-        <v>60</v>
-      </c>
-      <c r="F48" t="s">
+      <c r="G48" t="s">
         <v>242</v>
       </c>
-      <c r="G48" t="s">
+      <c r="H48" t="s">
         <v>243</v>
       </c>
-      <c r="H48" t="s">
+      <c r="I48" t="s">
         <v>244</v>
       </c>
-      <c r="I48" t="s">
+      <c r="J48" t="s">
         <v>245</v>
       </c>
-      <c r="J48" t="s">
+      <c r="K48" s="1" t="s">
         <v>246</v>
       </c>
-      <c r="K48" s="1" t="s">
-        <v>247</v>
-      </c>
-    </row>
-    <row r="49" spans="3:11" x14ac:dyDescent="0.2">
+    </row>
+    <row r="49" spans="3:11" x14ac:dyDescent="0.25">
       <c r="C49">
         <v>22</v>
       </c>
       <c r="D49" t="s">
+        <v>247</v>
+      </c>
+      <c r="E49" t="s">
+        <v>60</v>
+      </c>
+      <c r="F49" t="s">
         <v>248</v>
       </c>
-      <c r="E49" t="s">
-        <v>60</v>
-      </c>
-      <c r="F49" t="s">
+      <c r="G49" t="s">
         <v>249</v>
       </c>
-      <c r="G49" t="s">
+      <c r="H49" t="s">
         <v>250</v>
       </c>
-      <c r="H49" t="s">
+      <c r="I49" t="s">
         <v>251</v>
       </c>
-      <c r="I49" t="s">
+      <c r="J49" t="s">
         <v>252</v>
       </c>
-      <c r="J49" t="s">
+      <c r="K49" s="1" t="s">
         <v>253</v>
       </c>
-      <c r="K49" s="1" t="s">
-        <v>254</v>
-      </c>
-    </row>
-    <row r="50" spans="3:11" x14ac:dyDescent="0.2">
+    </row>
+    <row r="50" spans="3:11" x14ac:dyDescent="0.25">
       <c r="C50">
         <v>2</v>
       </c>
       <c r="D50" t="s">
+        <v>254</v>
+      </c>
+      <c r="E50" t="s">
+        <v>60</v>
+      </c>
+      <c r="F50" t="s">
         <v>255</v>
       </c>
-      <c r="E50" t="s">
-        <v>60</v>
-      </c>
-      <c r="F50" t="s">
+      <c r="G50" t="s">
         <v>256</v>
       </c>
-      <c r="G50" t="s">
+      <c r="H50" t="s">
         <v>257</v>
       </c>
-      <c r="H50" t="s">
+      <c r="I50" t="s">
         <v>258</v>
       </c>
-      <c r="I50" t="s">
+      <c r="J50" t="s">
         <v>259</v>
       </c>
-      <c r="J50" t="s">
-        <v>260</v>
-      </c>
       <c r="K50" s="1" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="51" spans="3:11" x14ac:dyDescent="0.2">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="51" spans="3:11" x14ac:dyDescent="0.25">
       <c r="C51">
         <v>13</v>
       </c>
       <c r="D51" t="s">
+        <v>260</v>
+      </c>
+      <c r="E51" t="s">
+        <v>60</v>
+      </c>
+      <c r="F51" t="s">
         <v>261</v>
       </c>
-      <c r="E51" t="s">
-        <v>60</v>
-      </c>
-      <c r="F51" t="s">
+      <c r="G51" t="s">
         <v>262</v>
       </c>
-      <c r="G51" t="s">
-        <v>263</v>
-      </c>
       <c r="H51" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="I51" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="J51" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="K51" s="1" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="52" spans="3:11" x14ac:dyDescent="0.2">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="52" spans="3:11" x14ac:dyDescent="0.25">
       <c r="C52">
         <v>38</v>
       </c>
       <c r="D52" t="s">
+        <v>263</v>
+      </c>
+      <c r="E52" t="s">
+        <v>60</v>
+      </c>
+      <c r="F52" t="s">
         <v>264</v>
       </c>
-      <c r="E52" t="s">
-        <v>60</v>
-      </c>
-      <c r="F52" t="s">
+      <c r="G52" t="s">
         <v>265</v>
       </c>
-      <c r="G52" t="s">
+      <c r="H52" t="s">
         <v>266</v>
       </c>
-      <c r="H52" t="s">
-        <v>267</v>
-      </c>
       <c r="I52" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="J52" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="K52" s="1" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
   </sheetData>

</xml_diff>